<commit_message>
Adjust for early return
</commit_message>
<xml_diff>
--- a/early_return_discovery/rental_car_booking2_columns.xlsx
+++ b/early_return_discovery/rental_car_booking2_columns.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\calla\Google Drive\Resume &amp; Stuff\ezhire\sql_analysis\mysql_queries\early_return_discovery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19519BB7-AE82-4051-8645-6DB929576E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3F02535-C691-4815-8235-0831D6BC1BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{96DC2DA1-DB1E-470B-98C3-37E52C0AAC59}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1474" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1899" uniqueCount="526">
   <si>
     <t>Field</t>
   </si>
@@ -1450,6 +1450,168 @@
   </si>
   <si>
     <t>Notes</t>
+  </si>
+  <si>
+    <t>use early return flag as the primary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">filter; ignore early return table </t>
+  </si>
+  <si>
+    <t>info if flag is 0</t>
+  </si>
+  <si>
+    <t>early return date</t>
+  </si>
+  <si>
+    <t>original return date</t>
+  </si>
+  <si>
+    <t>delivery date</t>
+  </si>
+  <si>
+    <t>extension days</t>
+  </si>
+  <si>
+    <t>initial days</t>
+  </si>
+  <si>
+    <t>RAEZ00063818</t>
+  </si>
+  <si>
+    <t>RAEZ00063686</t>
+  </si>
+  <si>
+    <t>RAEZ00063799</t>
+  </si>
+  <si>
+    <t>Monday</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>MotorKart Rent A Car LLC</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>Craig</t>
+  </si>
+  <si>
+    <t>Du</t>
+  </si>
+  <si>
+    <t>Vasanth Kumsr</t>
+  </si>
+  <si>
+    <t>Omar Farouk</t>
+  </si>
+  <si>
+    <t>Colquhoun</t>
+  </si>
+  <si>
+    <t>Lidan</t>
+  </si>
+  <si>
+    <t>Williams</t>
+  </si>
+  <si>
+    <t>Istaitie</t>
+  </si>
+  <si>
+    <t>vc4z8jr8p6@privaterelay.appleid.com</t>
+  </si>
+  <si>
+    <t>jjdu@hotmail.com</t>
+  </si>
+  <si>
+    <t>vwilliamscis@gmail.com</t>
+  </si>
+  <si>
+    <t>omarstaytieh@gmail.com</t>
+  </si>
+  <si>
+    <t>HatchBack</t>
+  </si>
+  <si>
+    <t>Featured</t>
+  </si>
+  <si>
+    <t>Kia Picanto or Similar</t>
+  </si>
+  <si>
+    <t>Hyundai Accent or Similar</t>
+  </si>
+  <si>
+    <t>Ciaz</t>
+  </si>
+  <si>
+    <t>Picanto</t>
+  </si>
+  <si>
+    <t>Accent</t>
+  </si>
+  <si>
+    <t>Kia</t>
+  </si>
+  <si>
+    <t>Hyundai</t>
+  </si>
+  <si>
+    <t>grey</t>
+  </si>
+  <si>
+    <t>Grey</t>
+  </si>
+  <si>
+    <t>silver</t>
+  </si>
+  <si>
+    <t>69V5+5H6 Dubai International Airport - Parking B - Airport Rd - opp. Terminal 3 - Garhoud - Dubai - United Arab Emirates</t>
+  </si>
+  <si>
+    <t>18 3 St - Springs 2 - Dubai - United Arab Emirates</t>
+  </si>
+  <si>
+    <t>4 10 St - Al Nad - Al Qasimia - Sharjah - United Arab Emirates</t>
+  </si>
+  <si>
+    <t>3643+Q49 - Jumeirah Village - Dubai - United Arab Emirates</t>
+  </si>
+  <si>
+    <t>58G4+CGF - Nad Al Sheba 1 - Dubai - United Arab Emirates</t>
+  </si>
+  <si>
+    <t>extension days set to 0</t>
+  </si>
+  <si>
+    <t>to avoid calculation</t>
+  </si>
+  <si>
+    <t>issues</t>
+  </si>
+  <si>
+    <t>since extension_days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">query pulled original </t>
+  </si>
+  <si>
+    <t>extension days not</t>
+  </si>
+  <si>
+    <t>extension after early return</t>
+  </si>
+  <si>
+    <t>as shown above</t>
+  </si>
+  <si>
+    <t>with extension days</t>
+  </si>
+  <si>
+    <t>&gt; total days</t>
   </si>
 </sst>
 </file>
@@ -1948,7 +2110,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1982,6 +2144,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -7462,15 +7627,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E38DF04-706C-45B9-823C-B1D363E215F7}">
-  <dimension ref="A1:E147"/>
+  <dimension ref="A1:L159"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.42578125" style="2" customWidth="1"/>
     <col min="2" max="2" width="33.140625" style="2" customWidth="1"/>
     <col min="3" max="5" width="29.28515625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="42.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.28515625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="17" style="2" customWidth="1"/>
+    <col min="9" max="9" width="19.28515625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="22.28515625" style="2" customWidth="1"/>
+    <col min="11" max="12" width="33.140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>266</v>
       </c>
@@ -7483,8 +7654,29 @@
       <c r="D1" s="11">
         <v>225443</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>266</v>
+      </c>
+      <c r="G1" s="11">
+        <v>30174</v>
+      </c>
+      <c r="H1" s="11">
+        <v>210299</v>
+      </c>
+      <c r="I1" s="11">
+        <v>240667</v>
+      </c>
+      <c r="J1" s="11">
+        <v>240709</v>
+      </c>
+      <c r="K1" s="11">
+        <v>240727</v>
+      </c>
+      <c r="L1" s="11">
+        <v>240755</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -7497,8 +7689,29 @@
       <c r="D2" s="2" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G2" s="2">
+        <v>1100042428</v>
+      </c>
+      <c r="H2" s="2">
+        <v>1100128258</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="K2" s="2">
+        <v>316</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>267</v>
       </c>
@@ -7512,8 +7725,29 @@
         <v>45231</v>
       </c>
       <c r="E3" s="6"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3" t="s">
+        <v>267</v>
+      </c>
+      <c r="G3" s="6">
+        <v>43984</v>
+      </c>
+      <c r="H3" s="6">
+        <v>45164</v>
+      </c>
+      <c r="I3" s="6">
+        <v>45292</v>
+      </c>
+      <c r="J3" s="6">
+        <v>45292</v>
+      </c>
+      <c r="K3" s="6">
+        <v>45292</v>
+      </c>
+      <c r="L3" s="6">
+        <v>45292</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>268</v>
       </c>
@@ -7527,8 +7761,29 @@
         <v>45231.531307870369</v>
       </c>
       <c r="E4" s="4"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" t="s">
+        <v>268</v>
+      </c>
+      <c r="G4" s="4">
+        <v>43984.320127314815</v>
+      </c>
+      <c r="H4" s="4">
+        <v>45164.936585648145</v>
+      </c>
+      <c r="I4" s="4">
+        <v>45292.009479166663</v>
+      </c>
+      <c r="J4" s="4">
+        <v>45292.448877314811</v>
+      </c>
+      <c r="K4" s="4">
+        <v>45292.479525462964</v>
+      </c>
+      <c r="L4" s="4">
+        <v>45292.534745370373</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>269</v>
       </c>
@@ -7542,8 +7797,29 @@
         <v>45434.202175925922</v>
       </c>
       <c r="E5" s="4"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5" t="s">
+        <v>269</v>
+      </c>
+      <c r="G5" s="4">
+        <v>45439.429768518516</v>
+      </c>
+      <c r="H5" s="4">
+        <v>45439.429768518516</v>
+      </c>
+      <c r="I5" s="4">
+        <v>45439.429768518516</v>
+      </c>
+      <c r="J5" s="4">
+        <v>45439.429768518516</v>
+      </c>
+      <c r="K5" s="4">
+        <v>45439.429768518516</v>
+      </c>
+      <c r="L5" s="4">
+        <v>45439.429768518516</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>270</v>
       </c>
@@ -7556,8 +7832,29 @@
       <c r="D6" s="2" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" t="s">
+        <v>270</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>272</v>
       </c>
@@ -7570,8 +7867,29 @@
       <c r="D7" s="2">
         <v>2023</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G7" s="2">
+        <v>2020</v>
+      </c>
+      <c r="H7" s="2">
+        <v>2023</v>
+      </c>
+      <c r="I7" s="2">
+        <v>2024</v>
+      </c>
+      <c r="J7" s="2">
+        <v>2024</v>
+      </c>
+      <c r="K7" s="2">
+        <v>2024</v>
+      </c>
+      <c r="L7" s="2">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>273</v>
       </c>
@@ -7584,8 +7902,29 @@
       <c r="D8" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8" t="s">
+        <v>273</v>
+      </c>
+      <c r="G8" s="2">
+        <v>2</v>
+      </c>
+      <c r="H8" s="2">
+        <v>3</v>
+      </c>
+      <c r="I8" s="2">
+        <v>1</v>
+      </c>
+      <c r="J8" s="2">
+        <v>1</v>
+      </c>
+      <c r="K8" s="2">
+        <v>1</v>
+      </c>
+      <c r="L8" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>274</v>
       </c>
@@ -7598,8 +7937,29 @@
       <c r="D9" s="2">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9" t="s">
+        <v>274</v>
+      </c>
+      <c r="G9" s="2">
+        <v>6</v>
+      </c>
+      <c r="H9" s="2">
+        <v>8</v>
+      </c>
+      <c r="I9" s="2">
+        <v>1</v>
+      </c>
+      <c r="J9" s="2">
+        <v>1</v>
+      </c>
+      <c r="K9" s="2">
+        <v>1</v>
+      </c>
+      <c r="L9" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>275</v>
       </c>
@@ -7612,8 +7972,29 @@
       <c r="D10" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10" t="s">
+        <v>275</v>
+      </c>
+      <c r="G10" s="2">
+        <v>2</v>
+      </c>
+      <c r="H10" s="2">
+        <v>26</v>
+      </c>
+      <c r="I10" s="2">
+        <v>1</v>
+      </c>
+      <c r="J10" s="2">
+        <v>1</v>
+      </c>
+      <c r="K10" s="2">
+        <v>1</v>
+      </c>
+      <c r="L10" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>276</v>
       </c>
@@ -7626,8 +8007,29 @@
       <c r="D11" s="2">
         <v>44</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11" t="s">
+        <v>276</v>
+      </c>
+      <c r="G11" s="2">
+        <v>23</v>
+      </c>
+      <c r="H11" s="2">
+        <v>34</v>
+      </c>
+      <c r="I11" s="2">
+        <v>1</v>
+      </c>
+      <c r="J11" s="2">
+        <v>1</v>
+      </c>
+      <c r="K11" s="2">
+        <v>1</v>
+      </c>
+      <c r="L11" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>277</v>
       </c>
@@ -7640,8 +8042,29 @@
       <c r="D12" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12" t="s">
+        <v>277</v>
+      </c>
+      <c r="G12" s="2">
+        <v>3</v>
+      </c>
+      <c r="H12" s="2">
+        <v>7</v>
+      </c>
+      <c r="I12" s="2">
+        <v>2</v>
+      </c>
+      <c r="J12" s="2">
+        <v>2</v>
+      </c>
+      <c r="K12" s="2">
+        <v>2</v>
+      </c>
+      <c r="L12" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>278</v>
       </c>
@@ -7654,8 +8077,29 @@
       <c r="D13" s="2" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13" t="s">
+        <v>278</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>280</v>
       </c>
@@ -7668,8 +8112,29 @@
       <c r="D14" s="2">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14" t="s">
+        <v>280</v>
+      </c>
+      <c r="G14" s="2">
+        <v>7</v>
+      </c>
+      <c r="H14" s="2">
+        <v>22</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0</v>
+      </c>
+      <c r="J14" s="2">
+        <v>10</v>
+      </c>
+      <c r="K14" s="2">
+        <v>11</v>
+      </c>
+      <c r="L14" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>281</v>
       </c>
@@ -7682,8 +8147,29 @@
       <c r="D15" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15" t="s">
+        <v>281</v>
+      </c>
+      <c r="G15" s="2">
+        <v>1</v>
+      </c>
+      <c r="H15" s="2">
+        <v>1</v>
+      </c>
+      <c r="I15" s="2">
+        <v>1</v>
+      </c>
+      <c r="J15" s="2">
+        <v>1</v>
+      </c>
+      <c r="K15" s="2">
+        <v>1</v>
+      </c>
+      <c r="L15" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>282</v>
       </c>
@@ -7696,23 +8182,65 @@
       <c r="D16" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="F16" t="s">
+        <v>282</v>
+      </c>
+      <c r="G16" s="2">
+        <v>1</v>
+      </c>
+      <c r="H16" s="2">
+        <v>1</v>
+      </c>
+      <c r="I16" s="2">
+        <v>1</v>
+      </c>
+      <c r="J16" s="2">
+        <v>1</v>
+      </c>
+      <c r="K16" s="2">
+        <v>1</v>
+      </c>
+      <c r="L16" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
         <v>283</v>
       </c>
-      <c r="B17" s="6">
+      <c r="B17" s="10">
         <v>43984</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="10">
         <v>45165</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="10">
         <v>45232</v>
       </c>
-      <c r="E17" s="6"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E17" s="10"/>
+      <c r="F17" t="s">
+        <v>283</v>
+      </c>
+      <c r="G17" s="10">
+        <v>43984</v>
+      </c>
+      <c r="H17" s="10">
+        <v>45165</v>
+      </c>
+      <c r="I17" s="10">
+        <v>45293</v>
+      </c>
+      <c r="J17" s="10">
+        <v>45292</v>
+      </c>
+      <c r="K17" s="10">
+        <v>45292</v>
+      </c>
+      <c r="L17" s="10">
+        <v>45292</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>284</v>
       </c>
@@ -7726,8 +8254,29 @@
         <v>45232.750694444447</v>
       </c>
       <c r="E18" s="4"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" t="s">
+        <v>284</v>
+      </c>
+      <c r="G18" s="4">
+        <v>43984.416666666664</v>
+      </c>
+      <c r="H18" s="4">
+        <v>45165.513888888891</v>
+      </c>
+      <c r="I18" s="4">
+        <v>45293.80972222222</v>
+      </c>
+      <c r="J18" s="4">
+        <v>45292.510416666664</v>
+      </c>
+      <c r="K18" s="4">
+        <v>45292.604166666664</v>
+      </c>
+      <c r="L18" s="4">
+        <v>45292.929166666669</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>285</v>
       </c>
@@ -7740,8 +8289,29 @@
       <c r="D19" s="2">
         <v>2023</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" t="s">
+        <v>285</v>
+      </c>
+      <c r="G19" s="2">
+        <v>2020</v>
+      </c>
+      <c r="H19" s="2">
+        <v>2023</v>
+      </c>
+      <c r="I19" s="2">
+        <v>2024</v>
+      </c>
+      <c r="J19" s="2">
+        <v>2024</v>
+      </c>
+      <c r="K19" s="2">
+        <v>2024</v>
+      </c>
+      <c r="L19" s="2">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>286</v>
       </c>
@@ -7754,8 +8324,29 @@
       <c r="D20" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" t="s">
+        <v>286</v>
+      </c>
+      <c r="G20" s="2">
+        <v>2</v>
+      </c>
+      <c r="H20" s="2">
+        <v>3</v>
+      </c>
+      <c r="I20" s="2">
+        <v>1</v>
+      </c>
+      <c r="J20" s="2">
+        <v>1</v>
+      </c>
+      <c r="K20" s="2">
+        <v>1</v>
+      </c>
+      <c r="L20" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>287</v>
       </c>
@@ -7768,8 +8359,29 @@
       <c r="D21" s="2">
         <v>11</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21" t="s">
+        <v>287</v>
+      </c>
+      <c r="G21" s="2">
+        <v>6</v>
+      </c>
+      <c r="H21" s="2">
+        <v>8</v>
+      </c>
+      <c r="I21" s="2">
+        <v>1</v>
+      </c>
+      <c r="J21" s="2">
+        <v>1</v>
+      </c>
+      <c r="K21" s="2">
+        <v>1</v>
+      </c>
+      <c r="L21" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>288</v>
       </c>
@@ -7782,8 +8394,29 @@
       <c r="D22" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22" t="s">
+        <v>288</v>
+      </c>
+      <c r="G22" s="2">
+        <v>2</v>
+      </c>
+      <c r="H22" s="2">
+        <v>27</v>
+      </c>
+      <c r="I22" s="2">
+        <v>2</v>
+      </c>
+      <c r="J22" s="2">
+        <v>1</v>
+      </c>
+      <c r="K22" s="2">
+        <v>1</v>
+      </c>
+      <c r="L22" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>289</v>
       </c>
@@ -7796,8 +8429,29 @@
       <c r="D23" s="2">
         <v>44</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23" t="s">
+        <v>289</v>
+      </c>
+      <c r="G23" s="2">
+        <v>23</v>
+      </c>
+      <c r="H23" s="2">
+        <v>34</v>
+      </c>
+      <c r="I23" s="2">
+        <v>1</v>
+      </c>
+      <c r="J23" s="2">
+        <v>1</v>
+      </c>
+      <c r="K23" s="2">
+        <v>1</v>
+      </c>
+      <c r="L23" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>290</v>
       </c>
@@ -7810,8 +8464,29 @@
       <c r="D24" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24" t="s">
+        <v>290</v>
+      </c>
+      <c r="G24" s="2">
+        <v>3</v>
+      </c>
+      <c r="H24" s="2">
+        <v>1</v>
+      </c>
+      <c r="I24" s="2">
+        <v>3</v>
+      </c>
+      <c r="J24" s="2">
+        <v>2</v>
+      </c>
+      <c r="K24" s="2">
+        <v>2</v>
+      </c>
+      <c r="L24" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>291</v>
       </c>
@@ -7824,8 +8499,29 @@
       <c r="D25" s="2" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25" t="s">
+        <v>291</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>293</v>
       </c>
@@ -7838,8 +8534,29 @@
       <c r="D26" s="2">
         <v>18</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26" t="s">
+        <v>293</v>
+      </c>
+      <c r="G26" s="2">
+        <v>10</v>
+      </c>
+      <c r="H26" s="2">
+        <v>12</v>
+      </c>
+      <c r="I26" s="2">
+        <v>19</v>
+      </c>
+      <c r="J26" s="2">
+        <v>12</v>
+      </c>
+      <c r="K26" s="2">
+        <v>14</v>
+      </c>
+      <c r="L26" s="2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -7853,8 +8570,29 @@
         <v>45511</v>
       </c>
       <c r="E27" s="6"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27" t="s">
+        <v>158</v>
+      </c>
+      <c r="G27" s="6">
+        <v>0</v>
+      </c>
+      <c r="H27" s="6">
+        <v>1</v>
+      </c>
+      <c r="I27" s="6">
+        <v>0</v>
+      </c>
+      <c r="J27" s="6">
+        <v>1</v>
+      </c>
+      <c r="K27" s="6">
+        <v>1</v>
+      </c>
+      <c r="L27" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>294</v>
       </c>
@@ -7870,8 +8608,29 @@
       <c r="E28" s="10" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F28" t="s">
+        <v>53</v>
+      </c>
+      <c r="G28" s="10">
+        <v>44044</v>
+      </c>
+      <c r="H28" s="10">
+        <v>45194</v>
+      </c>
+      <c r="I28" s="10">
+        <v>45417</v>
+      </c>
+      <c r="J28" s="10">
+        <v>45353</v>
+      </c>
+      <c r="K28" s="10">
+        <v>45311</v>
+      </c>
+      <c r="L28" s="10">
+        <v>45303</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>295</v>
       </c>
@@ -7884,8 +8643,29 @@
       <c r="D29" s="2">
         <v>2024</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29" t="s">
+        <v>294</v>
+      </c>
+      <c r="G29" s="2">
+        <v>44044.375</v>
+      </c>
+      <c r="H29" s="2">
+        <v>45194.729166666664</v>
+      </c>
+      <c r="I29" s="2">
+        <v>45417.828472222223</v>
+      </c>
+      <c r="J29" s="2">
+        <v>45353.6875</v>
+      </c>
+      <c r="K29" s="2">
+        <v>45311.416666666664</v>
+      </c>
+      <c r="L29" s="2">
+        <v>45303.833333333336</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>296</v>
       </c>
@@ -7898,8 +8678,29 @@
       <c r="D30" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30" t="s">
+        <v>295</v>
+      </c>
+      <c r="G30" s="2">
+        <v>2020</v>
+      </c>
+      <c r="H30" s="2">
+        <v>2023</v>
+      </c>
+      <c r="I30" s="2">
+        <v>2024</v>
+      </c>
+      <c r="J30" s="2">
+        <v>2024</v>
+      </c>
+      <c r="K30" s="2">
+        <v>2024</v>
+      </c>
+      <c r="L30" s="2">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>297</v>
       </c>
@@ -7912,8 +8713,29 @@
       <c r="D31" s="2">
         <v>8</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F31" t="s">
+        <v>296</v>
+      </c>
+      <c r="G31" s="2">
+        <v>3</v>
+      </c>
+      <c r="H31" s="2">
+        <v>3</v>
+      </c>
+      <c r="I31" s="2">
+        <v>2</v>
+      </c>
+      <c r="J31" s="2">
+        <v>1</v>
+      </c>
+      <c r="K31" s="2">
+        <v>1</v>
+      </c>
+      <c r="L31" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>298</v>
       </c>
@@ -7926,8 +8748,29 @@
       <c r="D32" s="2">
         <v>7</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F32" t="s">
+        <v>297</v>
+      </c>
+      <c r="G32" s="2">
+        <v>8</v>
+      </c>
+      <c r="H32" s="2">
+        <v>9</v>
+      </c>
+      <c r="I32" s="2">
+        <v>5</v>
+      </c>
+      <c r="J32" s="2">
+        <v>3</v>
+      </c>
+      <c r="K32" s="2">
+        <v>1</v>
+      </c>
+      <c r="L32" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>299</v>
       </c>
@@ -7940,8 +8783,29 @@
       <c r="D33" s="2">
         <v>32</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33" t="s">
+        <v>298</v>
+      </c>
+      <c r="G33" s="2">
+        <v>1</v>
+      </c>
+      <c r="H33" s="2">
+        <v>25</v>
+      </c>
+      <c r="I33" s="2">
+        <v>5</v>
+      </c>
+      <c r="J33" s="2">
+        <v>2</v>
+      </c>
+      <c r="K33" s="2">
+        <v>20</v>
+      </c>
+      <c r="L33" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>300</v>
       </c>
@@ -7954,8 +8818,29 @@
       <c r="D34" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F34" t="s">
+        <v>299</v>
+      </c>
+      <c r="G34" s="2">
+        <v>30</v>
+      </c>
+      <c r="H34" s="2">
+        <v>39</v>
+      </c>
+      <c r="I34" s="2">
+        <v>18</v>
+      </c>
+      <c r="J34" s="2">
+        <v>8</v>
+      </c>
+      <c r="K34" s="2">
+        <v>2</v>
+      </c>
+      <c r="L34" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>301</v>
       </c>
@@ -7968,8 +8853,29 @@
       <c r="D35" s="2" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F35" t="s">
+        <v>300</v>
+      </c>
+      <c r="G35" s="2">
+        <v>7</v>
+      </c>
+      <c r="H35" s="2">
+        <v>2</v>
+      </c>
+      <c r="I35" s="2">
+        <v>1</v>
+      </c>
+      <c r="J35" s="2">
+        <v>7</v>
+      </c>
+      <c r="K35" s="2">
+        <v>7</v>
+      </c>
+      <c r="L35" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>302</v>
       </c>
@@ -7982,8 +8888,29 @@
       <c r="D36" s="2">
         <v>18</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F36" t="s">
+        <v>301</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>303</v>
       </c>
@@ -7996,8 +8923,29 @@
       <c r="D37" s="2" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37" t="s">
+        <v>302</v>
+      </c>
+      <c r="G37" s="2">
+        <v>9</v>
+      </c>
+      <c r="H37" s="2">
+        <v>17</v>
+      </c>
+      <c r="I37" s="2">
+        <v>19</v>
+      </c>
+      <c r="J37" s="2">
+        <v>16</v>
+      </c>
+      <c r="K37" s="2">
+        <v>10</v>
+      </c>
+      <c r="L37" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>305</v>
       </c>
@@ -8010,8 +8958,29 @@
       <c r="D38" s="2" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F38" t="s">
+        <v>303</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>307</v>
       </c>
@@ -8024,8 +8993,29 @@
       <c r="D39" s="2" t="s">
         <v>308</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39" t="s">
+        <v>305</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="L39" s="2" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>309</v>
       </c>
@@ -8038,8 +9028,29 @@
       <c r="D40" s="2" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40" t="s">
+        <v>307</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>311</v>
       </c>
@@ -8052,8 +9063,29 @@
       <c r="D41" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F41" t="s">
+        <v>309</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>312</v>
       </c>
@@ -8066,8 +9098,29 @@
       <c r="D42" s="2" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F42" t="s">
+        <v>311</v>
+      </c>
+      <c r="G42" s="2">
+        <v>0</v>
+      </c>
+      <c r="H42" s="2">
+        <v>1</v>
+      </c>
+      <c r="I42" s="2">
+        <v>1</v>
+      </c>
+      <c r="J42" s="2">
+        <v>0</v>
+      </c>
+      <c r="K42" s="2">
+        <v>0</v>
+      </c>
+      <c r="L42" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>313</v>
       </c>
@@ -8080,8 +9133,29 @@
       <c r="D43" s="2" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F43" t="s">
+        <v>312</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>315</v>
       </c>
@@ -8094,8 +9168,29 @@
       <c r="D44" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F44" t="s">
+        <v>313</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>316</v>
       </c>
@@ -8108,8 +9203,29 @@
       <c r="D45" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F45" t="s">
+        <v>315</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>317</v>
       </c>
@@ -8122,8 +9238,29 @@
       <c r="D46" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F46" t="s">
+        <v>316</v>
+      </c>
+      <c r="G46" s="2">
+        <v>0</v>
+      </c>
+      <c r="H46" s="2">
+        <v>0</v>
+      </c>
+      <c r="I46" s="2">
+        <v>0</v>
+      </c>
+      <c r="J46" s="2">
+        <v>0</v>
+      </c>
+      <c r="K46" s="2">
+        <v>0</v>
+      </c>
+      <c r="L46" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>318</v>
       </c>
@@ -8136,8 +9273,29 @@
       <c r="D47" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F47" t="s">
+        <v>317</v>
+      </c>
+      <c r="G47" s="2">
+        <v>0</v>
+      </c>
+      <c r="H47" s="2">
+        <v>0</v>
+      </c>
+      <c r="I47" s="2">
+        <v>0</v>
+      </c>
+      <c r="J47" s="2">
+        <v>0</v>
+      </c>
+      <c r="K47" s="2">
+        <v>0</v>
+      </c>
+      <c r="L47" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
         <v>30</v>
       </c>
@@ -8153,8 +9311,29 @@
       <c r="E48" s="3" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F48" t="s">
+        <v>318</v>
+      </c>
+      <c r="G48" s="3">
+        <v>0</v>
+      </c>
+      <c r="H48" s="3">
+        <v>0</v>
+      </c>
+      <c r="I48" s="3">
+        <v>0</v>
+      </c>
+      <c r="J48" s="3">
+        <v>0</v>
+      </c>
+      <c r="K48" s="3">
+        <v>0</v>
+      </c>
+      <c r="L48" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>320</v>
       </c>
@@ -8167,8 +9346,29 @@
       <c r="D49" s="2" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F49" t="s">
+        <v>30</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="L49" s="2" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>322</v>
       </c>
@@ -8181,8 +9381,29 @@
       <c r="D50" s="2" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F50" t="s">
+        <v>320</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="L50" s="2" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>324</v>
       </c>
@@ -8195,8 +9416,29 @@
       <c r="D51" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F51" t="s">
+        <v>322</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="L51" s="2" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>325</v>
       </c>
@@ -8209,8 +9451,29 @@
       <c r="D52" s="2" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F52" t="s">
+        <v>324</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="L52" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>327</v>
       </c>
@@ -8223,8 +9486,29 @@
       <c r="D53" s="2" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F53" t="s">
+        <v>325</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>328</v>
       </c>
@@ -8237,8 +9521,29 @@
       <c r="D54" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F54" t="s">
+        <v>327</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="L54" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>329</v>
       </c>
@@ -8251,13 +9556,55 @@
       <c r="D55" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F55" t="s">
+        <v>328</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L55" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F56" t="s">
+        <v>329</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>331</v>
       </c>
@@ -8270,8 +9617,11 @@
       <c r="D57" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F57" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>332</v>
       </c>
@@ -8284,8 +9634,29 @@
       <c r="D58" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F58" t="s">
+        <v>331</v>
+      </c>
+      <c r="G58" s="2">
+        <v>1</v>
+      </c>
+      <c r="H58" s="2">
+        <v>1</v>
+      </c>
+      <c r="I58" s="2">
+        <v>2</v>
+      </c>
+      <c r="J58" s="2">
+        <v>4</v>
+      </c>
+      <c r="K58" s="2">
+        <v>1</v>
+      </c>
+      <c r="L58" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>333</v>
       </c>
@@ -8298,8 +9669,29 @@
       <c r="D59" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F59" t="s">
+        <v>332</v>
+      </c>
+      <c r="G59" s="2">
+        <v>0</v>
+      </c>
+      <c r="H59" s="2">
+        <v>0</v>
+      </c>
+      <c r="I59" s="2">
+        <v>0</v>
+      </c>
+      <c r="J59" s="2">
+        <v>0</v>
+      </c>
+      <c r="K59" s="2">
+        <v>0</v>
+      </c>
+      <c r="L59" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>334</v>
       </c>
@@ -8312,8 +9704,29 @@
       <c r="D60" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F60" t="s">
+        <v>333</v>
+      </c>
+      <c r="G60" s="2">
+        <v>1</v>
+      </c>
+      <c r="H60" s="2">
+        <v>1</v>
+      </c>
+      <c r="I60" s="2">
+        <v>2</v>
+      </c>
+      <c r="J60" s="2">
+        <v>4</v>
+      </c>
+      <c r="K60" s="2">
+        <v>1</v>
+      </c>
+      <c r="L60" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>335</v>
       </c>
@@ -8326,8 +9739,29 @@
       <c r="D61" s="2">
         <v>519820</v>
       </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F61" t="s">
+        <v>334</v>
+      </c>
+      <c r="G61" s="2">
+        <v>0</v>
+      </c>
+      <c r="H61" s="2">
+        <v>0</v>
+      </c>
+      <c r="I61" s="2">
+        <v>0</v>
+      </c>
+      <c r="J61" s="2">
+        <v>0</v>
+      </c>
+      <c r="K61" s="2">
+        <v>0</v>
+      </c>
+      <c r="L61" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>336</v>
       </c>
@@ -8340,8 +9774,29 @@
       <c r="D62" s="2" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F62" t="s">
+        <v>335</v>
+      </c>
+      <c r="G62" s="2">
+        <v>62218</v>
+      </c>
+      <c r="H62" s="2">
+        <v>499829</v>
+      </c>
+      <c r="I62" s="2">
+        <v>450413</v>
+      </c>
+      <c r="J62" s="2">
+        <v>365396</v>
+      </c>
+      <c r="K62" s="2">
+        <v>549342</v>
+      </c>
+      <c r="L62" s="2">
+        <v>3661</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>338</v>
       </c>
@@ -8354,8 +9809,29 @@
       <c r="D63" s="2" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F63" t="s">
+        <v>336</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="K63" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="L63" s="2" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>340</v>
       </c>
@@ -8368,8 +9844,29 @@
       <c r="D64" s="2" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F64" t="s">
+        <v>338</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="H64" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="K64" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="L64" s="2" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>342</v>
       </c>
@@ -8383,8 +9880,29 @@
         <v>33787</v>
       </c>
       <c r="E65" s="6"/>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F65" t="s">
+        <v>340</v>
+      </c>
+      <c r="G65" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="H65" s="6" t="s">
+        <v>443</v>
+      </c>
+      <c r="I65" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="J65" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="K65" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="L65" s="6" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>343</v>
       </c>
@@ -8397,8 +9915,29 @@
       <c r="D66" s="2">
         <v>32</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F66" t="s">
+        <v>342</v>
+      </c>
+      <c r="G66" s="2">
+        <v>33787</v>
+      </c>
+      <c r="H66" s="2">
+        <v>34700</v>
+      </c>
+      <c r="I66" s="2">
+        <v>33787</v>
+      </c>
+      <c r="J66" s="2">
+        <v>43831</v>
+      </c>
+      <c r="K66" s="2">
+        <v>33787</v>
+      </c>
+      <c r="L66" s="2">
+        <v>43831</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>344</v>
       </c>
@@ -8411,8 +9950,29 @@
       <c r="D67" s="2" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F67" t="s">
+        <v>343</v>
+      </c>
+      <c r="G67" s="2">
+        <v>32</v>
+      </c>
+      <c r="H67" s="2">
+        <v>29</v>
+      </c>
+      <c r="I67" s="2">
+        <v>32</v>
+      </c>
+      <c r="J67" s="2">
+        <v>4</v>
+      </c>
+      <c r="K67" s="2">
+        <v>32</v>
+      </c>
+      <c r="L67" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>346</v>
       </c>
@@ -8425,8 +9985,29 @@
       <c r="D68" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F68" t="s">
+        <v>344</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="J68" s="2">
+        <v>0</v>
+      </c>
+      <c r="K68" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="L68" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>24</v>
       </c>
@@ -8439,8 +10020,29 @@
       <c r="D69" s="3">
         <v>279</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F69" t="s">
+        <v>346</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K69" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L69" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>347</v>
       </c>
@@ -8453,8 +10055,29 @@
       <c r="D70" s="3">
         <v>151</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F70" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G70" s="3">
+        <v>60</v>
+      </c>
+      <c r="H70" s="3">
+        <v>29</v>
+      </c>
+      <c r="I70" s="3">
+        <v>124</v>
+      </c>
+      <c r="J70" s="12">
+        <v>61</v>
+      </c>
+      <c r="K70" s="12">
+        <v>19</v>
+      </c>
+      <c r="L70" s="12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>348</v>
       </c>
@@ -8467,8 +10090,29 @@
       <c r="D71" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F71" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="G71" s="3">
+        <v>30</v>
+      </c>
+      <c r="H71" s="3">
+        <v>0</v>
+      </c>
+      <c r="I71" s="3">
+        <v>94</v>
+      </c>
+      <c r="J71" s="12">
+        <v>32</v>
+      </c>
+      <c r="K71" s="12">
+        <v>25</v>
+      </c>
+      <c r="L71" s="12">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>349</v>
       </c>
@@ -8481,8 +10125,29 @@
       <c r="D72" s="2">
         <v>46.63</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F72" s="8" t="s">
+        <v>348</v>
+      </c>
+      <c r="G72" s="3">
+        <v>0</v>
+      </c>
+      <c r="H72" s="3">
+        <v>142.72</v>
+      </c>
+      <c r="I72" s="3">
+        <v>0</v>
+      </c>
+      <c r="J72" s="3">
+        <v>47.61</v>
+      </c>
+      <c r="K72" s="3">
+        <v>0</v>
+      </c>
+      <c r="L72" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>350</v>
       </c>
@@ -8495,8 +10160,29 @@
       <c r="D73" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F73" t="s">
+        <v>349</v>
+      </c>
+      <c r="G73" s="2">
+        <v>33.299999237060497</v>
+      </c>
+      <c r="H73" s="2">
+        <v>98.43</v>
+      </c>
+      <c r="I73" s="2">
+        <v>53.299999237060497</v>
+      </c>
+      <c r="J73" s="2">
+        <v>47.61</v>
+      </c>
+      <c r="K73" s="2">
+        <v>99.85</v>
+      </c>
+      <c r="L73" s="2">
+        <v>114.14</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>351</v>
       </c>
@@ -8509,8 +10195,29 @@
       <c r="D74" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F74" t="s">
+        <v>350</v>
+      </c>
+      <c r="G74" s="2">
+        <v>6.17</v>
+      </c>
+      <c r="H74" s="2">
+        <v>0</v>
+      </c>
+      <c r="I74" s="2">
+        <v>0</v>
+      </c>
+      <c r="J74" s="2">
+        <v>5</v>
+      </c>
+      <c r="K74" s="2">
+        <v>0</v>
+      </c>
+      <c r="L74" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>352</v>
       </c>
@@ -8523,8 +10230,29 @@
       <c r="D75" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F75" t="s">
+        <v>351</v>
+      </c>
+      <c r="G75" s="2">
+        <v>0</v>
+      </c>
+      <c r="H75" s="2">
+        <v>0</v>
+      </c>
+      <c r="I75" s="2">
+        <v>0</v>
+      </c>
+      <c r="J75" s="2">
+        <v>0</v>
+      </c>
+      <c r="K75" s="2">
+        <v>0</v>
+      </c>
+      <c r="L75" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>353</v>
       </c>
@@ -8537,8 +10265,29 @@
       <c r="D76" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F76" t="s">
+        <v>352</v>
+      </c>
+      <c r="G76" s="2">
+        <v>0</v>
+      </c>
+      <c r="H76" s="2">
+        <v>0</v>
+      </c>
+      <c r="I76" s="2">
+        <v>0</v>
+      </c>
+      <c r="J76" s="2">
+        <v>0</v>
+      </c>
+      <c r="K76" s="2">
+        <v>0</v>
+      </c>
+      <c r="L76" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>354</v>
       </c>
@@ -8551,8 +10300,29 @@
       <c r="D77" s="2" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F77" t="s">
+        <v>353</v>
+      </c>
+      <c r="G77" s="2">
+        <v>0</v>
+      </c>
+      <c r="H77" s="2">
+        <v>0</v>
+      </c>
+      <c r="I77" s="2">
+        <v>0</v>
+      </c>
+      <c r="J77" s="2">
+        <v>0</v>
+      </c>
+      <c r="K77" s="2">
+        <v>0</v>
+      </c>
+      <c r="L77" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>356</v>
       </c>
@@ -8565,8 +10335,29 @@
       <c r="D78" s="2">
         <v>51.3</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F78" t="s">
+        <v>354</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="H78" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="I78" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="J78" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="K78" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="L78" s="2" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>357</v>
       </c>
@@ -8579,8 +10370,29 @@
       <c r="D79" s="2" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F79" t="s">
+        <v>356</v>
+      </c>
+      <c r="G79" s="2">
+        <v>0</v>
+      </c>
+      <c r="H79" s="2">
+        <v>56.63</v>
+      </c>
+      <c r="I79" s="2">
+        <v>53.3</v>
+      </c>
+      <c r="J79" s="2">
+        <v>56.63</v>
+      </c>
+      <c r="K79" s="2">
+        <v>53.3</v>
+      </c>
+      <c r="L79" s="2">
+        <v>63.3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>359</v>
       </c>
@@ -8593,8 +10405,29 @@
       <c r="D80" s="2">
         <v>13009.77</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F80" t="s">
+        <v>357</v>
+      </c>
+      <c r="G80" s="2">
+        <v>0</v>
+      </c>
+      <c r="H80" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="I80" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="J80" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="K80" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="L80" s="2" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>360</v>
       </c>
@@ -8607,8 +10440,29 @@
       <c r="D81" s="2">
         <v>5868.64013671875</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F81" t="s">
+        <v>359</v>
+      </c>
+      <c r="G81" s="2">
+        <v>1998</v>
+      </c>
+      <c r="H81" s="2">
+        <v>2854.47</v>
+      </c>
+      <c r="I81" s="2">
+        <v>6609.2</v>
+      </c>
+      <c r="J81" s="2">
+        <v>2904.21</v>
+      </c>
+      <c r="K81" s="2">
+        <v>1897.15</v>
+      </c>
+      <c r="L81" s="2">
+        <v>1255.54</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>361</v>
       </c>
@@ -8621,8 +10475,29 @@
       <c r="D82" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F82" t="s">
+        <v>360</v>
+      </c>
+      <c r="G82" s="2">
+        <v>998.99997711181595</v>
+      </c>
+      <c r="H82" s="2">
+        <v>2854.47</v>
+      </c>
+      <c r="I82" s="2">
+        <v>1598.99997711181</v>
+      </c>
+      <c r="J82" s="2">
+        <v>1380.69</v>
+      </c>
+      <c r="K82" s="2">
+        <v>-599.099999999999</v>
+      </c>
+      <c r="L82" s="2">
+        <v>-1369.68</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>362</v>
       </c>
@@ -8635,8 +10510,29 @@
       <c r="D83" s="2">
         <v>39</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F83" t="s">
+        <v>361</v>
+      </c>
+      <c r="G83" s="2">
+        <v>0</v>
+      </c>
+      <c r="H83" s="2">
+        <v>142.72</v>
+      </c>
+      <c r="I83" s="2">
+        <v>0</v>
+      </c>
+      <c r="J83" s="2">
+        <v>47.61</v>
+      </c>
+      <c r="K83" s="2">
+        <v>0</v>
+      </c>
+      <c r="L83" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>363</v>
       </c>
@@ -8649,8 +10545,29 @@
       <c r="D84" s="2">
         <v>39</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F84" t="s">
+        <v>362</v>
+      </c>
+      <c r="G84" s="2">
+        <v>39</v>
+      </c>
+      <c r="H84" s="2">
+        <v>39</v>
+      </c>
+      <c r="I84" s="2">
+        <v>29</v>
+      </c>
+      <c r="J84" s="2">
+        <v>39</v>
+      </c>
+      <c r="K84" s="2">
+        <v>39</v>
+      </c>
+      <c r="L84" s="2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>364</v>
       </c>
@@ -8663,8 +10580,29 @@
       <c r="D85" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F85" t="s">
+        <v>363</v>
+      </c>
+      <c r="G85" s="2">
+        <v>39</v>
+      </c>
+      <c r="H85" s="2">
+        <v>39</v>
+      </c>
+      <c r="I85" s="2">
+        <v>39</v>
+      </c>
+      <c r="J85" s="2">
+        <v>39</v>
+      </c>
+      <c r="K85" s="2">
+        <v>39</v>
+      </c>
+      <c r="L85" s="2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>365</v>
       </c>
@@ -8677,8 +10615,29 @@
       <c r="D86" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F86" t="s">
+        <v>364</v>
+      </c>
+      <c r="G86" s="2">
+        <v>0</v>
+      </c>
+      <c r="H86" s="2">
+        <v>0</v>
+      </c>
+      <c r="I86" s="2">
+        <v>0</v>
+      </c>
+      <c r="J86" s="2">
+        <v>0</v>
+      </c>
+      <c r="K86" s="2">
+        <v>0</v>
+      </c>
+      <c r="L86" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>366</v>
       </c>
@@ -8691,8 +10650,29 @@
       <c r="D87" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F87" t="s">
+        <v>365</v>
+      </c>
+      <c r="G87" s="2">
+        <v>370.2</v>
+      </c>
+      <c r="H87" s="2">
+        <v>0</v>
+      </c>
+      <c r="I87" s="2">
+        <v>0</v>
+      </c>
+      <c r="J87" s="2">
+        <v>305</v>
+      </c>
+      <c r="K87" s="2">
+        <v>0</v>
+      </c>
+      <c r="L87" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>367</v>
       </c>
@@ -8705,8 +10685,29 @@
       <c r="D88" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F88" t="s">
+        <v>366</v>
+      </c>
+      <c r="G88" s="2">
+        <v>0</v>
+      </c>
+      <c r="H88" s="2">
+        <v>0</v>
+      </c>
+      <c r="I88" s="2">
+        <v>0</v>
+      </c>
+      <c r="J88" s="2">
+        <v>0</v>
+      </c>
+      <c r="K88" s="2">
+        <v>0</v>
+      </c>
+      <c r="L88" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>368</v>
       </c>
@@ -8719,8 +10720,29 @@
       <c r="D89" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F89" t="s">
+        <v>367</v>
+      </c>
+      <c r="G89" s="2">
+        <v>0</v>
+      </c>
+      <c r="H89" s="2">
+        <v>0</v>
+      </c>
+      <c r="I89" s="2">
+        <v>0</v>
+      </c>
+      <c r="J89" s="2">
+        <v>0</v>
+      </c>
+      <c r="K89" s="2">
+        <v>0</v>
+      </c>
+      <c r="L89" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>369</v>
       </c>
@@ -8733,8 +10755,29 @@
       <c r="D90" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F90" t="s">
+        <v>368</v>
+      </c>
+      <c r="G90" s="2">
+        <v>0</v>
+      </c>
+      <c r="H90" s="2">
+        <v>0</v>
+      </c>
+      <c r="I90" s="2">
+        <v>0</v>
+      </c>
+      <c r="J90" s="2">
+        <v>0</v>
+      </c>
+      <c r="K90" s="2">
+        <v>0</v>
+      </c>
+      <c r="L90" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>370</v>
       </c>
@@ -8747,8 +10790,29 @@
       <c r="D91" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F91" t="s">
+        <v>369</v>
+      </c>
+      <c r="G91" s="2">
+        <v>0</v>
+      </c>
+      <c r="H91" s="2">
+        <v>0</v>
+      </c>
+      <c r="I91" s="2">
+        <v>0</v>
+      </c>
+      <c r="J91" s="2">
+        <v>0</v>
+      </c>
+      <c r="K91" s="2">
+        <v>0</v>
+      </c>
+      <c r="L91" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>371</v>
       </c>
@@ -8761,8 +10825,29 @@
       <c r="D92" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F92" t="s">
+        <v>370</v>
+      </c>
+      <c r="G92" s="2">
+        <v>0</v>
+      </c>
+      <c r="H92" s="2">
+        <v>0</v>
+      </c>
+      <c r="I92" s="2">
+        <v>0</v>
+      </c>
+      <c r="J92" s="2">
+        <v>0</v>
+      </c>
+      <c r="K92" s="2">
+        <v>0</v>
+      </c>
+      <c r="L92" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>372</v>
       </c>
@@ -8775,8 +10860,29 @@
       <c r="D93" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F93" t="s">
+        <v>371</v>
+      </c>
+      <c r="G93" s="2">
+        <v>0</v>
+      </c>
+      <c r="H93" s="2">
+        <v>0</v>
+      </c>
+      <c r="I93" s="2">
+        <v>0</v>
+      </c>
+      <c r="J93" s="2">
+        <v>0</v>
+      </c>
+      <c r="K93" s="2">
+        <v>0</v>
+      </c>
+      <c r="L93" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>373</v>
       </c>
@@ -8789,8 +10895,29 @@
       <c r="D94" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F94" t="s">
+        <v>372</v>
+      </c>
+      <c r="G94" s="2">
+        <v>0</v>
+      </c>
+      <c r="H94" s="2">
+        <v>0</v>
+      </c>
+      <c r="I94" s="2">
+        <v>0</v>
+      </c>
+      <c r="J94" s="2">
+        <v>0</v>
+      </c>
+      <c r="K94" s="2">
+        <v>0</v>
+      </c>
+      <c r="L94" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>374</v>
       </c>
@@ -8803,8 +10930,29 @@
       <c r="D95" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F95" t="s">
+        <v>373</v>
+      </c>
+      <c r="G95" s="2">
+        <v>0</v>
+      </c>
+      <c r="H95" s="2">
+        <v>0</v>
+      </c>
+      <c r="I95" s="2">
+        <v>0</v>
+      </c>
+      <c r="J95" s="2">
+        <v>0</v>
+      </c>
+      <c r="K95" s="2">
+        <v>0</v>
+      </c>
+      <c r="L95" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>375</v>
       </c>
@@ -8817,8 +10965,29 @@
       <c r="D96" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F96" t="s">
+        <v>374</v>
+      </c>
+      <c r="G96" s="2">
+        <v>0</v>
+      </c>
+      <c r="H96" s="2">
+        <v>0</v>
+      </c>
+      <c r="I96" s="2">
+        <v>0</v>
+      </c>
+      <c r="J96" s="2">
+        <v>0</v>
+      </c>
+      <c r="K96" s="2">
+        <v>0</v>
+      </c>
+      <c r="L96" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>376</v>
       </c>
@@ -8831,8 +11000,29 @@
       <c r="D97" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F97" t="s">
+        <v>375</v>
+      </c>
+      <c r="G97" s="2">
+        <v>370.2</v>
+      </c>
+      <c r="H97" s="3">
+        <v>0</v>
+      </c>
+      <c r="I97" s="2">
+        <v>0</v>
+      </c>
+      <c r="J97" s="2">
+        <v>305</v>
+      </c>
+      <c r="K97" s="2">
+        <v>0</v>
+      </c>
+      <c r="L97" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>377</v>
       </c>
@@ -8845,8 +11035,29 @@
       <c r="D98" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F98" t="s">
+        <v>376</v>
+      </c>
+      <c r="G98" s="2">
+        <v>0</v>
+      </c>
+      <c r="H98" s="3">
+        <v>0</v>
+      </c>
+      <c r="I98" s="2">
+        <v>0</v>
+      </c>
+      <c r="J98" s="2">
+        <v>0</v>
+      </c>
+      <c r="K98" s="2">
+        <v>0</v>
+      </c>
+      <c r="L98" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>378</v>
       </c>
@@ -8859,8 +11070,29 @@
       <c r="D99" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F99" t="s">
+        <v>377</v>
+      </c>
+      <c r="G99" s="2">
+        <v>0</v>
+      </c>
+      <c r="H99" s="2">
+        <v>0</v>
+      </c>
+      <c r="I99" s="2">
+        <v>0</v>
+      </c>
+      <c r="J99" s="2">
+        <v>0</v>
+      </c>
+      <c r="K99" s="2">
+        <v>0</v>
+      </c>
+      <c r="L99" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>379</v>
       </c>
@@ -8873,8 +11105,29 @@
       <c r="D100" s="2">
         <v>953.20349999999996</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F100" t="s">
+        <v>378</v>
+      </c>
+      <c r="G100" s="2">
+        <v>0</v>
+      </c>
+      <c r="H100" s="2">
+        <v>0</v>
+      </c>
+      <c r="I100" s="2">
+        <v>0</v>
+      </c>
+      <c r="J100" s="2">
+        <v>0</v>
+      </c>
+      <c r="K100" s="2">
+        <v>0</v>
+      </c>
+      <c r="L100" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>380</v>
       </c>
@@ -8887,8 +11140,29 @@
       <c r="D101" s="2">
         <v>3586.3935000000001</v>
       </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F101" t="s">
+        <v>379</v>
+      </c>
+      <c r="G101" s="2">
+        <v>122.31</v>
+      </c>
+      <c r="H101" s="2">
+        <v>0</v>
+      </c>
+      <c r="I101" s="2">
+        <v>333.85999999999899</v>
+      </c>
+      <c r="J101" s="2">
+        <v>0</v>
+      </c>
+      <c r="K101" s="2">
+        <v>0</v>
+      </c>
+      <c r="L101" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>381</v>
       </c>
@@ -8901,8 +11175,29 @@
       <c r="D102" s="2">
         <v>13087.77</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F102" t="s">
+        <v>380</v>
+      </c>
+      <c r="G102" s="2">
+        <v>499.719999999999</v>
+      </c>
+      <c r="H102" s="2">
+        <v>0</v>
+      </c>
+      <c r="I102" s="2">
+        <v>333.85999999999899</v>
+      </c>
+      <c r="J102" s="2">
+        <v>0</v>
+      </c>
+      <c r="K102" s="2">
+        <v>0</v>
+      </c>
+      <c r="L102" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>382</v>
       </c>
@@ -8915,8 +11210,29 @@
       <c r="D103" s="2">
         <v>12987.77</v>
       </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F103" t="s">
+        <v>381</v>
+      </c>
+      <c r="G103" s="2">
+        <v>2446.1999999999998</v>
+      </c>
+      <c r="H103" s="2">
+        <v>3075.19</v>
+      </c>
+      <c r="I103" s="2">
+        <v>6677.2</v>
+      </c>
+      <c r="J103" s="2">
+        <v>3334.82</v>
+      </c>
+      <c r="K103" s="2">
+        <v>1975.15</v>
+      </c>
+      <c r="L103" s="2">
+        <v>1333.54</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A104" s="8" t="s">
         <v>383</v>
       </c>
@@ -8932,8 +11248,29 @@
       <c r="E104" s="3" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F104" t="s">
+        <v>382</v>
+      </c>
+      <c r="G104" s="3">
+        <v>2446.1999999999998</v>
+      </c>
+      <c r="H104" s="12">
+        <v>3075.19</v>
+      </c>
+      <c r="I104" s="3">
+        <v>6677.2</v>
+      </c>
+      <c r="J104" s="3">
+        <v>3334.82</v>
+      </c>
+      <c r="K104" s="3">
+        <v>1975.15</v>
+      </c>
+      <c r="L104" s="3">
+        <v>1333.54</v>
+      </c>
+    </row>
+    <row r="105" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A105" s="8" t="s">
         <v>384</v>
       </c>
@@ -8949,8 +11286,29 @@
       <c r="E105" s="3" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F105" t="s">
+        <v>383</v>
+      </c>
+      <c r="G105" s="3">
+        <v>2446.1999999999998</v>
+      </c>
+      <c r="H105" s="12">
+        <v>3075.19</v>
+      </c>
+      <c r="I105" s="3">
+        <v>6677.2</v>
+      </c>
+      <c r="J105" s="3">
+        <v>3334.82</v>
+      </c>
+      <c r="K105" s="3">
+        <v>1975.15</v>
+      </c>
+      <c r="L105" s="3">
+        <v>1333.54</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>385</v>
       </c>
@@ -8963,8 +11321,29 @@
       <c r="D106" s="2">
         <v>6046.6398387146</v>
       </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F106" t="s">
+        <v>384</v>
+      </c>
+      <c r="G106" s="2">
+        <v>2446.1999999999998</v>
+      </c>
+      <c r="H106" s="2">
+        <v>3075.19</v>
+      </c>
+      <c r="I106" s="2">
+        <v>6677.2</v>
+      </c>
+      <c r="J106" s="2">
+        <v>3334.82</v>
+      </c>
+      <c r="K106" s="2">
+        <v>1975.15</v>
+      </c>
+      <c r="L106" s="2">
+        <v>1333.54</v>
+      </c>
+    </row>
+    <row r="107" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A107" s="8" t="s">
         <v>386</v>
       </c>
@@ -8980,8 +11359,29 @@
       <c r="E107" s="3" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F107" t="s">
+        <v>385</v>
+      </c>
+      <c r="G107" s="3">
+        <v>1262.1000228881801</v>
+      </c>
+      <c r="H107" s="3">
+        <v>3075.19</v>
+      </c>
+      <c r="I107" s="3">
+        <v>1667.0000717163</v>
+      </c>
+      <c r="J107" s="3">
+        <v>1651.3</v>
+      </c>
+      <c r="K107" s="3">
+        <v>-521.099999999999</v>
+      </c>
+      <c r="L107" s="3">
+        <v>-1291.6799999999901</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A108" s="8" t="s">
         <v>387</v>
       </c>
@@ -8997,8 +11397,29 @@
       <c r="E108" s="3" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F108" t="s">
+        <v>386</v>
+      </c>
+      <c r="G108" s="3">
+        <v>1262.1000228881801</v>
+      </c>
+      <c r="H108" s="3">
+        <v>3075.19</v>
+      </c>
+      <c r="I108" s="3">
+        <v>1667.0000717163</v>
+      </c>
+      <c r="J108" s="3">
+        <v>1651.3</v>
+      </c>
+      <c r="K108" s="3">
+        <v>-521.099999999999</v>
+      </c>
+      <c r="L108" s="3">
+        <v>-1291.6799999999901</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>388</v>
       </c>
@@ -9011,8 +11432,29 @@
       <c r="D109" s="2">
         <v>5946.6398387146</v>
       </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F109" t="s">
+        <v>387</v>
+      </c>
+      <c r="G109" s="2">
+        <v>1262.1000228881801</v>
+      </c>
+      <c r="H109" s="2">
+        <v>3075.19</v>
+      </c>
+      <c r="I109" s="2">
+        <v>1667.0000717163</v>
+      </c>
+      <c r="J109" s="2">
+        <v>1651.3</v>
+      </c>
+      <c r="K109" s="2">
+        <v>-521.099999999999</v>
+      </c>
+      <c r="L109" s="2">
+        <v>-1291.6799999999901</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>389</v>
       </c>
@@ -9025,8 +11467,29 @@
       <c r="D110" s="2">
         <v>13087.77</v>
       </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F110" t="s">
+        <v>388</v>
+      </c>
+      <c r="G110" s="2">
+        <v>1262.1000228881801</v>
+      </c>
+      <c r="H110" s="2">
+        <v>3075.19</v>
+      </c>
+      <c r="I110" s="2">
+        <v>1667.0000717163</v>
+      </c>
+      <c r="J110" s="2">
+        <v>1651.3</v>
+      </c>
+      <c r="K110" s="2">
+        <v>-521.099999999999</v>
+      </c>
+      <c r="L110" s="2">
+        <v>-1291.6799999999901</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>390</v>
       </c>
@@ -9039,8 +11502,29 @@
       <c r="D111" s="2">
         <v>3586.3935000000001</v>
       </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F111" t="s">
+        <v>389</v>
+      </c>
+      <c r="G111" s="2">
+        <v>2446.1999999999998</v>
+      </c>
+      <c r="H111" s="2">
+        <v>3075.19</v>
+      </c>
+      <c r="I111" s="2">
+        <v>6677.2</v>
+      </c>
+      <c r="J111" s="2">
+        <v>3334.82</v>
+      </c>
+      <c r="K111" s="2">
+        <v>1975.15</v>
+      </c>
+      <c r="L111" s="2">
+        <v>1333.54</v>
+      </c>
+    </row>
+    <row r="112" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A112" s="8" t="s">
         <v>391</v>
       </c>
@@ -9056,8 +11540,29 @@
       <c r="E112" s="3" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F112" t="s">
+        <v>390</v>
+      </c>
+      <c r="G112" s="3">
+        <v>499.719999999999</v>
+      </c>
+      <c r="H112" s="3">
+        <v>0</v>
+      </c>
+      <c r="I112" s="3">
+        <v>333.85999999999899</v>
+      </c>
+      <c r="J112" s="3">
+        <v>0</v>
+      </c>
+      <c r="K112" s="3">
+        <v>0</v>
+      </c>
+      <c r="L112" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>392</v>
       </c>
@@ -9070,8 +11575,29 @@
       <c r="D113" s="2">
         <v>7041.1301612854004</v>
       </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F113" t="s">
+        <v>391</v>
+      </c>
+      <c r="G113" s="2">
+        <v>1184.0999771118099</v>
+      </c>
+      <c r="H113" s="2">
+        <v>0</v>
+      </c>
+      <c r="I113" s="2">
+        <v>5010.1999282836896</v>
+      </c>
+      <c r="J113" s="3">
+        <v>1683.52</v>
+      </c>
+      <c r="K113" s="3">
+        <v>2496.25</v>
+      </c>
+      <c r="L113" s="3">
+        <v>2625.22</v>
+      </c>
+    </row>
+    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>393</v>
       </c>
@@ -9084,8 +11610,29 @@
       <c r="D114" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F114" t="s">
+        <v>392</v>
+      </c>
+      <c r="G114" s="2">
+        <v>1184.0999771118099</v>
+      </c>
+      <c r="H114" s="2">
+        <v>0</v>
+      </c>
+      <c r="I114" s="2">
+        <v>5010.1999282836896</v>
+      </c>
+      <c r="J114" s="3">
+        <v>1683.52</v>
+      </c>
+      <c r="K114" s="3">
+        <v>2496.25</v>
+      </c>
+      <c r="L114" s="3">
+        <v>2625.22</v>
+      </c>
+    </row>
+    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>394</v>
       </c>
@@ -9098,13 +11645,55 @@
       <c r="D115" s="2" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F115" t="s">
+        <v>393</v>
+      </c>
+      <c r="G115" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H115" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I115" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J115" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K115" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L115" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F116" t="s">
+        <v>394</v>
+      </c>
+      <c r="G116" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H116" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I116" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J116" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K116" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L116" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>396</v>
       </c>
@@ -9118,8 +11707,17 @@
         <v>45183.472962962966</v>
       </c>
       <c r="E117" s="4"/>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F117" t="s">
+        <v>395</v>
+      </c>
+      <c r="G117" s="4"/>
+      <c r="H117" s="4"/>
+      <c r="I117" s="4"/>
+      <c r="J117" s="4"/>
+      <c r="K117" s="4"/>
+      <c r="L117" s="4"/>
+    </row>
+    <row r="118" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>397</v>
       </c>
@@ -9129,8 +11727,29 @@
       <c r="D118" s="2" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F118" t="s">
+        <v>396</v>
+      </c>
+      <c r="G118" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H118" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="I118" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="J118" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="K118" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="L118" s="2">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>398</v>
       </c>
@@ -9143,8 +11762,26 @@
       <c r="D119" s="2">
         <v>286</v>
       </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F119" t="s">
+        <v>397</v>
+      </c>
+      <c r="G119" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I119" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J119" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K119" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L119" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>399</v>
       </c>
@@ -9157,8 +11794,29 @@
       <c r="D120" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F120" t="s">
+        <v>398</v>
+      </c>
+      <c r="G120" s="2">
+        <v>77</v>
+      </c>
+      <c r="H120" s="2">
+        <v>259</v>
+      </c>
+      <c r="I120" s="2">
+        <v>286</v>
+      </c>
+      <c r="J120" s="2">
+        <v>439</v>
+      </c>
+      <c r="K120" s="2">
+        <v>95</v>
+      </c>
+      <c r="L120" s="2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>400</v>
       </c>
@@ -9171,8 +11829,29 @@
       <c r="D121" s="2" t="s">
         <v>401</v>
       </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F121" t="s">
+        <v>399</v>
+      </c>
+      <c r="G121" s="2">
+        <v>1</v>
+      </c>
+      <c r="H121" s="2">
+        <v>2</v>
+      </c>
+      <c r="I121" s="2">
+        <v>2</v>
+      </c>
+      <c r="J121" s="2">
+        <v>1</v>
+      </c>
+      <c r="K121" s="2">
+        <v>2</v>
+      </c>
+      <c r="L121" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>402</v>
       </c>
@@ -9185,8 +11864,29 @@
       <c r="D122" s="2" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F122" t="s">
+        <v>400</v>
+      </c>
+      <c r="G122" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="H122" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="I122" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="J122" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="K122" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="L122" s="2" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>404</v>
       </c>
@@ -9199,8 +11899,29 @@
       <c r="D123" s="2" t="s">
         <v>405</v>
       </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F123" t="s">
+        <v>402</v>
+      </c>
+      <c r="G123" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="H123" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="I123" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="J123" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="K123" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="L123" s="2" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>406</v>
       </c>
@@ -9213,8 +11934,29 @@
       <c r="D124" s="2" t="s">
         <v>407</v>
       </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F124" t="s">
+        <v>404</v>
+      </c>
+      <c r="G124" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="H124" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="I124" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="J124" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="K124" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="L124" s="2" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>408</v>
       </c>
@@ -9227,8 +11969,29 @@
       <c r="D125" s="2" t="s">
         <v>409</v>
       </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F125" t="s">
+        <v>406</v>
+      </c>
+      <c r="G125" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="H125" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I125" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="J125" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="K125" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="L125" s="2" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>410</v>
       </c>
@@ -9241,8 +12004,29 @@
       <c r="D126" s="2" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F126" t="s">
+        <v>408</v>
+      </c>
+      <c r="G126" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H126" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I126" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="J126" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="K126" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="L126" s="2" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>411</v>
       </c>
@@ -9255,8 +12039,29 @@
       <c r="D127" s="2" t="s">
         <v>412</v>
       </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F127" t="s">
+        <v>410</v>
+      </c>
+      <c r="G127" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="H127" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="I127" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="J127" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="K127" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="L127" s="2" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>413</v>
       </c>
@@ -9269,8 +12074,29 @@
       <c r="D128" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F128" t="s">
+        <v>411</v>
+      </c>
+      <c r="G128" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="H128" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="I128" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="J128" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="K128" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="L128" s="2" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>68</v>
       </c>
@@ -9283,8 +12109,29 @@
       <c r="D129" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F129" t="s">
+        <v>413</v>
+      </c>
+      <c r="G129" s="2">
+        <v>1</v>
+      </c>
+      <c r="H129" s="2">
+        <v>1</v>
+      </c>
+      <c r="I129" s="2">
+        <v>1</v>
+      </c>
+      <c r="J129" s="2">
+        <v>1</v>
+      </c>
+      <c r="K129" s="2">
+        <v>1</v>
+      </c>
+      <c r="L129" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>48</v>
       </c>
@@ -9297,8 +12144,29 @@
       <c r="D130" s="2" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F130" t="s">
+        <v>68</v>
+      </c>
+      <c r="G130" s="2">
+        <v>1</v>
+      </c>
+      <c r="H130" s="2">
+        <v>3</v>
+      </c>
+      <c r="I130" s="2">
+        <v>1</v>
+      </c>
+      <c r="J130" s="2">
+        <v>1</v>
+      </c>
+      <c r="K130" s="2">
+        <v>3</v>
+      </c>
+      <c r="L130" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>414</v>
       </c>
@@ -9311,8 +12179,29 @@
       <c r="D131" s="2" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F131" t="s">
+        <v>48</v>
+      </c>
+      <c r="G131" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="H131" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="I131" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="J131" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="K131" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="L131" s="2" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>416</v>
       </c>
@@ -9325,8 +12214,29 @@
       <c r="D132" s="2">
         <v>24.470874879371902</v>
       </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F132" t="s">
+        <v>414</v>
+      </c>
+      <c r="G132" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="H132" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="I132" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="J132" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="K132" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="L132" s="2" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>417</v>
       </c>
@@ -9339,8 +12249,29 @@
       <c r="D133" s="2">
         <v>54.3728211522102</v>
       </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F133" t="s">
+        <v>416</v>
+      </c>
+      <c r="G133" s="2">
+        <v>25.207868490199999</v>
+      </c>
+      <c r="H133" s="2">
+        <v>25.3991525</v>
+      </c>
+      <c r="I133" s="2">
+        <v>25.243100199999901</v>
+      </c>
+      <c r="J133" s="2">
+        <v>25.057747299999999</v>
+      </c>
+      <c r="K133" s="2">
+        <v>25.341177425777001</v>
+      </c>
+      <c r="L133" s="2">
+        <v>25.0562629988571</v>
+      </c>
+    </row>
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>58</v>
       </c>
@@ -9353,8 +12284,29 @@
       <c r="D134" s="2" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F134" t="s">
+        <v>417</v>
+      </c>
+      <c r="G134" s="2">
+        <v>55.294146873099997</v>
+      </c>
+      <c r="H134" s="2">
+        <v>55.4374702</v>
+      </c>
+      <c r="I134" s="2">
+        <v>55.358893999999999</v>
+      </c>
+      <c r="J134" s="2">
+        <v>55.166035000000001</v>
+      </c>
+      <c r="K134" s="2">
+        <v>55.390896834433001</v>
+      </c>
+      <c r="L134" s="2">
+        <v>55.203684847853303</v>
+      </c>
+    </row>
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>418</v>
       </c>
@@ -9367,8 +12319,29 @@
       <c r="D135" s="2" t="s">
         <v>419</v>
       </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F135" t="s">
+        <v>58</v>
+      </c>
+      <c r="G135" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="H135" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="I135" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="J135" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="K135" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="L135" s="2" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>420</v>
       </c>
@@ -9381,8 +12354,29 @@
       <c r="D136" s="2">
         <v>24.436384757738999</v>
       </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F136" t="s">
+        <v>418</v>
+      </c>
+      <c r="G136" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="H136" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I136" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="J136" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="K136" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="L136" s="2" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>421</v>
       </c>
@@ -9395,8 +12389,29 @@
       <c r="D137" s="2">
         <v>54.418286606669398</v>
       </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F137" t="s">
+        <v>420</v>
+      </c>
+      <c r="G137" s="2">
+        <v>25.204849237091299</v>
+      </c>
+      <c r="H137" s="2">
+        <v>25.3991525</v>
+      </c>
+      <c r="I137" s="2">
+        <v>25.1760625</v>
+      </c>
+      <c r="J137" s="2">
+        <v>25.057747299999999</v>
+      </c>
+      <c r="K137" s="2">
+        <v>25.341125874965101</v>
+      </c>
+      <c r="L137" s="2">
+        <v>25.0562629988571</v>
+      </c>
+    </row>
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>422</v>
       </c>
@@ -9409,8 +12424,29 @@
       <c r="D138" s="2">
         <v>8</v>
       </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F138" t="s">
+        <v>421</v>
+      </c>
+      <c r="G138" s="2">
+        <v>55.270782820880399</v>
+      </c>
+      <c r="H138" s="2">
+        <v>55.4374702</v>
+      </c>
+      <c r="I138" s="2">
+        <v>55.306312499999997</v>
+      </c>
+      <c r="J138" s="2">
+        <v>55.166035000000001</v>
+      </c>
+      <c r="K138" s="2">
+        <v>55.391204583764399</v>
+      </c>
+      <c r="L138" s="2">
+        <v>55.203684847853303</v>
+      </c>
+    </row>
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>423</v>
       </c>
@@ -9423,8 +12459,52 @@
       <c r="D139" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F139" t="s">
+        <v>422</v>
+      </c>
+      <c r="G139" s="2">
+        <v>2</v>
+      </c>
+      <c r="H139" s="2">
+        <v>1</v>
+      </c>
+      <c r="I139" s="2">
+        <v>5</v>
+      </c>
+      <c r="J139" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K139" s="2">
+        <v>10</v>
+      </c>
+      <c r="L139" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F140" t="s">
+        <v>423</v>
+      </c>
+      <c r="G140" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H140" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I140" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J140" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K140" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L140" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>471</v>
       </c>
@@ -9437,8 +12517,20 @@
       <c r="D141" s="11" t="s">
         <v>461</v>
       </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G141" s="11"/>
+      <c r="H141" s="11"/>
+      <c r="I141" s="11"/>
+      <c r="J141" s="13" t="s">
+        <v>516</v>
+      </c>
+      <c r="K141" s="13" t="s">
+        <v>516</v>
+      </c>
+      <c r="L141" s="13" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B142" s="3" t="s">
         <v>458</v>
       </c>
@@ -9448,8 +12540,20 @@
       <c r="D142" s="3" t="s">
         <v>467</v>
       </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G142" s="3"/>
+      <c r="H142" s="3"/>
+      <c r="I142" s="3"/>
+      <c r="J142" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="K142" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="L142" s="3" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B143" s="3" t="s">
         <v>459</v>
       </c>
@@ -9459,8 +12563,20 @@
       <c r="D143" s="3" t="s">
         <v>466</v>
       </c>
-    </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G143" s="3"/>
+      <c r="H143" s="3"/>
+      <c r="I143" s="3"/>
+      <c r="J143" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="K143" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="L143" s="3" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B144" s="3" t="s">
         <v>460</v>
       </c>
@@ -9468,8 +12584,20 @@
         <v>464</v>
       </c>
       <c r="D144" s="3"/>
-    </row>
-    <row r="145" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="G144" s="3"/>
+      <c r="H144" s="3"/>
+      <c r="I144" s="3"/>
+      <c r="J144" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="K144" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="L144" s="3" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="145" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B145" s="3"/>
       <c r="C145" s="3" t="s">
         <v>465</v>
@@ -9477,20 +12605,174 @@
       <c r="D145" s="3" t="s">
         <v>468</v>
       </c>
-    </row>
-    <row r="146" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="G145" s="3"/>
+      <c r="H145" s="3"/>
+      <c r="I145" s="3"/>
+      <c r="J145" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="K145" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="L145" s="3" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="146" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B146" s="3"/>
       <c r="C146" s="3"/>
       <c r="D146" s="3" t="s">
         <v>469</v>
       </c>
-    </row>
-    <row r="147" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="G146" s="3"/>
+      <c r="H146" s="3"/>
+      <c r="I146" s="3"/>
+      <c r="J146" s="3" t="s">
+        <v>521</v>
+      </c>
+      <c r="K146" s="3" t="s">
+        <v>521</v>
+      </c>
+      <c r="L146" s="3" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="147" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B147" s="3"/>
       <c r="C147" s="3"/>
       <c r="D147" s="3" t="s">
         <v>470</v>
       </c>
+      <c r="G147" s="3"/>
+      <c r="H147" s="3"/>
+      <c r="I147" s="3"/>
+      <c r="J147" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="K147" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="L147" s="3" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="148" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B148" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="G148" s="3"/>
+      <c r="H148" s="3"/>
+      <c r="I148" s="3"/>
+      <c r="J148" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="K148" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="L148" s="3" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="149" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B149" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="G149" s="3"/>
+      <c r="H149" s="3"/>
+      <c r="I149" s="3"/>
+      <c r="J149" s="3" t="s">
+        <v>524</v>
+      </c>
+      <c r="K149" s="3" t="s">
+        <v>524</v>
+      </c>
+      <c r="L149" s="3" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="150" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B150" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="G150" s="3"/>
+      <c r="H150" s="3"/>
+      <c r="I150" s="3"/>
+      <c r="J150" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="K150" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="L150" s="3" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="151" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C151" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="D151" s="6">
+        <v>45232</v>
+      </c>
+    </row>
+    <row r="152" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C152" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="D152" s="6">
+        <v>45390</v>
+      </c>
+      <c r="E152" s="2">
+        <f>D152-D151</f>
+        <v>158</v>
+      </c>
+    </row>
+    <row r="153" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C153" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="D153" s="6">
+        <v>45511</v>
+      </c>
+      <c r="E153" s="2">
+        <f>D153-D151</f>
+        <v>279</v>
+      </c>
+    </row>
+    <row r="155" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C155" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D155" s="2">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="156" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C156" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="D156" s="2">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="157" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C157" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="D157" s="2">
+        <f>D155-D156</f>
+        <v>128</v>
+      </c>
+      <c r="E157" s="6">
+        <f>D151+D157</f>
+        <v>45360</v>
+      </c>
+    </row>
+    <row r="159" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D159" s="2">
+        <f>E152-D157</f>
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>